<commit_message>
Add grobid client and processing of references
</commit_message>
<xml_diff>
--- a/data/refs.xlsx
+++ b/data/refs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\mariambzd\repos\bibMining\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F413E3D-4B82-44E0-AED1-A6BA33F7E902}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8413AC32-95C8-4D0A-BCBC-D3E16116F69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{377650F8-19B9-4377-A4DA-035DFD494C6A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="RAW" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RAW!$A$1:$L$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">RAW!$A$1:$M$30</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="220">
   <si>
     <t>Year</t>
   </si>
@@ -669,13 +669,43 @@
   </si>
   <si>
     <t>Synthesis of Small-Scale Mining Community Flood Vulnerability and Resilience Strategy in Ghana.pdf.tei</t>
+  </si>
+  <si>
+    <t>old_TeiFile</t>
+  </si>
+  <si>
+    <t>Investigating how climate changeadaptation can be incorporated into mine closure and rehabilitation strategies to strengthen social-ecological resilience</t>
+  </si>
+  <si>
+    <t>Mining community resilience explored through sustainable community development and perceptions of community wellbeing</t>
+  </si>
+  <si>
+    <t>An Inclusive Approach to Disaster Risk Reduction in Water-Related Hazards for the Mining Industry: Prioritizing the Multi-Dimensional Risk Framework for Achieving Sustainable Development</t>
+  </si>
+  <si>
+    <t>Landslide risk, resilience and resistance: confronting community resilience with economic benefits in landslide-prone areas in Kerala</t>
+  </si>
+  <si>
+    <t>Qi no tu i baba ni qwali (living down by the river): Impacts of flooding and mining on ecosystems and livelihoods</t>
+  </si>
+  <si>
+    <t>Lessons learned from flash floods early warning system in a mountainous rur-urban region of Colombia</t>
+  </si>
+  <si>
+    <t>Desalination in Chile's mining regions: Global drivers and local impacts of a technological fix to hydrosocial conflict</t>
+  </si>
+  <si>
+    <t>DISASTER GOVERNANCE AND COMMUNITY RESILIENCE: THE LAW AND THE ROLE OF SDMAs</t>
+  </si>
+  <si>
+    <t>Social innovation, ecological crises and creating mining host community resilience in Southern Africa</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -729,6 +759,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -750,7 +793,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -765,6 +808,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1099,7 +1147,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F6EBB6-5C58-44AD-B342-EE74F3AC3D94}">
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" style="7" customWidth="1"/>
@@ -1112,9 +1160,10 @@
     <col min="9" max="9" width="7.33203125" customWidth="1"/>
     <col min="10" max="10" width="14.109375" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="15" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
@@ -1146,13 +1195,16 @@
         <v>94</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>185</v>
       </c>
@@ -1186,11 +1238,14 @@
       <c r="K2" t="s">
         <v>186</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="M2" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>43</v>
       </c>
@@ -1224,11 +1279,14 @@
       <c r="K3" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="L3" t="s">
+      <c r="L3" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>90</v>
       </c>
@@ -1256,11 +1314,14 @@
       <c r="K4" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="L4" t="s">
+      <c r="L4" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="M4" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
@@ -1294,11 +1355,14 @@
       <c r="K5" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="M5" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>53</v>
       </c>
@@ -1332,11 +1396,14 @@
       <c r="K6" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="M6" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>14</v>
       </c>
@@ -1367,11 +1434,14 @@
       <c r="K7" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="M7" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="8" t="s">
         <v>79</v>
       </c>
@@ -1405,11 +1475,14 @@
       <c r="K8" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>121</v>
       </c>
@@ -1440,11 +1513,14 @@
       <c r="K9" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="10" t="s">
+        <v>217</v>
+      </c>
+      <c r="M9" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="8" t="s">
         <v>32</v>
       </c>
@@ -1478,11 +1554,14 @@
       <c r="K10" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="M10" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>190</v>
       </c>
@@ -1513,11 +1592,14 @@
       <c r="K11" t="s">
         <v>194</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="M11" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>116</v>
       </c>
@@ -1551,11 +1633,14 @@
       <c r="K12" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="M12" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
@@ -1589,11 +1674,14 @@
       <c r="K13" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="L13" t="s">
+      <c r="L13" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M13" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="7" t="s">
         <v>112</v>
       </c>
@@ -1624,11 +1712,14 @@
       <c r="K14" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="10" t="s">
+        <v>112</v>
+      </c>
+      <c r="M14" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>108</v>
       </c>
@@ -1659,11 +1750,14 @@
       <c r="K15" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="M15" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
         <v>54</v>
       </c>
@@ -1697,11 +1791,14 @@
       <c r="K16" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="M16" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>36</v>
       </c>
@@ -1735,11 +1832,14 @@
       <c r="K17" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="M17" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>55</v>
       </c>
@@ -1773,11 +1873,14 @@
       <c r="K18" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="L18" t="s">
+      <c r="L18" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>22</v>
       </c>
@@ -1802,11 +1905,14 @@
       <c r="K19" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L19" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="M19" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>25</v>
       </c>
@@ -1840,11 +1946,14 @@
       <c r="K20" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="L20" t="s">
+      <c r="L20" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="M20" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="8" t="s">
         <v>42</v>
       </c>
@@ -1878,11 +1987,14 @@
       <c r="K21" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="L21" t="s">
+      <c r="L21" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="M21" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="8" t="s">
         <v>84</v>
       </c>
@@ -1916,11 +2028,14 @@
       <c r="K22" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="L22" t="s">
+      <c r="L22" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="M22" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>126</v>
       </c>
@@ -1954,11 +2069,14 @@
       <c r="K23" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="L23" t="s">
+      <c r="L23" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="M23" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>30</v>
       </c>
@@ -1986,11 +2104,14 @@
       <c r="K24" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="L24" t="s">
+      <c r="L24" s="11" t="s">
+        <v>212</v>
+      </c>
+      <c r="M24" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>18</v>
       </c>
@@ -2024,11 +2145,14 @@
       <c r="K25" s="4" t="s">
         <v>143</v>
       </c>
-      <c r="L25" t="s">
+      <c r="L25" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="M25" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>196</v>
       </c>
@@ -2059,11 +2183,14 @@
       <c r="K26" t="s">
         <v>198</v>
       </c>
-      <c r="L26" t="s">
+      <c r="L26" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="M26" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>181</v>
       </c>
@@ -2097,11 +2224,14 @@
       <c r="K27" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L27" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="M27" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="8" t="s">
         <v>49</v>
       </c>
@@ -2135,11 +2265,14 @@
       <c r="K28" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="L28" t="s">
+      <c r="L28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="M28" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>206</v>
       </c>
@@ -2167,11 +2300,14 @@
       <c r="K29" t="s">
         <v>209</v>
       </c>
-      <c r="L29" t="s">
+      <c r="L29" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="M29" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
         <v>48</v>
       </c>
@@ -2205,13 +2341,16 @@
       <c r="K30" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="L30" t="s">
+      <c r="L30" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="M30" t="s">
         <v>167</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L30" xr:uid="{89F6EBB6-5C58-44AD-B342-EE74F3AC3D94}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L30">
+  <autoFilter ref="A1:M30" xr:uid="{89F6EBB6-5C58-44AD-B342-EE74F3AC3D94}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M30">
       <sortCondition ref="A1:A30"/>
     </sortState>
   </autoFilter>

</xml_diff>